<commit_message>
Refresh Feishu dashboard with solution GA4 data
</commit_message>
<xml_diff>
--- a/exports/feishu-base-import/seeed_解决方案增长_多维表格导入.xlsx
+++ b/exports/feishu-base-import/seeed_解决方案增长_多维表格导入.xlsx
@@ -159,7 +159,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>44310</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -179,7 +179,7 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>GA4未命中：需确认 seeed.cc / 中文站是否接入当前 GA4 Property，或下一次用 /solutions 过滤专项拉数</t>
+          <t>有可观察流量：建议按渠道和页面继续下钻</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
@@ -216,7 +216,7 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>0/12</t>
+          <t>12/12</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -273,7 +273,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>0.00</t>
+          <t>31.90</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -293,7 +293,7 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>GA4未命中</t>
+          <t>互动时间正常，可继续按页面主题细分判断</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
@@ -330,7 +330,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>840</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -350,7 +350,7 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>GA4未命中</t>
+          <t>转化处于可优化区间，建议做渠道和页面拆解</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
@@ -486,22 +486,22 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>23657</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>8824</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>0.00</t>
+          <t>34.84</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>0.00%</t>
+          <t>88.38%</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
@@ -511,22 +511,22 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>387</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>未命中</t>
+          <t>Email</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>GA4未命中</t>
+          <t>GA4已命中</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>GA4未命中：需确认 seeed.cc / 中文站是否接入当前 GA4 Property，或下一次用 /solutions 过滤专项拉数</t>
+          <t>有可观察流量：建议按渠道和页面继续下钻</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
@@ -573,47 +573,47 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>2.50</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>100.00%</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>待接入 CTA 点击事件</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
           <t>0</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>0.00</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>0.00%</t>
-        </is>
-      </c>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>待接入 CTA 点击事件</t>
-        </is>
-      </c>
-      <c r="L3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>未命中</t>
+          <t>Paid Search</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>GA4未命中</t>
+          <t>GA4已命中</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>GA4未命中：需确认 seeed.cc / 中文站是否接入当前 GA4 Property，或下一次用 /solutions 过滤专项拉数</t>
+          <t>样本偏少：先确认埋点和入口曝光，再判断增长</t>
         </is>
       </c>
       <c r="P3" t="inlineStr">
@@ -660,47 +660,47 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
+          <t>126</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>57</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>17.57</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>85.51%</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>待接入 CTA 点击事件</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
           <t>0</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>0.00</t>
-        </is>
-      </c>
-      <c r="J4" t="inlineStr">
-        <is>
-          <t>0.00%</t>
-        </is>
-      </c>
-      <c r="K4" t="inlineStr">
-        <is>
-          <t>待接入 CTA 点击事件</t>
-        </is>
-      </c>
-      <c r="L4" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>未命中</t>
+          <t>Direct</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>GA4未命中</t>
+          <t>GA4已命中</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>GA4未命中：需确认 seeed.cc / 中文站是否接入当前 GA4 Property，或下一次用 /solutions 过滤专项拉数</t>
+          <t>有流量但转化偏弱：优先检查CTA、表单入口和案例承接</t>
         </is>
       </c>
       <c r="P4" t="inlineStr">
@@ -747,22 +747,22 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1529</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>682</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>0.00</t>
+          <t>55.21</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>0.00%</t>
+          <t>86.24%</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
@@ -772,22 +772,22 @@
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>未命中</t>
+          <t>Organic Search</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>GA4未命中</t>
+          <t>GA4已命中</t>
         </is>
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>GA4未命中：需确认 seeed.cc / 中文站是否接入当前 GA4 Property，或下一次用 /solutions 过滤专项拉数</t>
+          <t>有流量但转化偏弱：优先检查CTA、表单入口和案例承接</t>
         </is>
       </c>
       <c r="P5" t="inlineStr">
@@ -834,22 +834,22 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>18536</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>7133</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>0.00</t>
+          <t>26.40</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>0.00%</t>
+          <t>80.99%</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
@@ -859,22 +859,22 @@
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>451</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>未命中</t>
+          <t>Referral</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>GA4未命中</t>
+          <t>GA4已命中</t>
         </is>
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>GA4未命中：需确认 seeed.cc / 中文站是否接入当前 GA4 Property，或下一次用 /solutions 过滤专项拉数</t>
+          <t>有可观察流量：建议按渠道和页面继续下钻</t>
         </is>
       </c>
       <c r="P6" t="inlineStr">
@@ -921,22 +921,22 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>259</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>142</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>0.00</t>
+          <t>20.32</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>0.00%</t>
+          <t>90.00%</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
@@ -946,22 +946,22 @@
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>未命中</t>
+          <t>Organic Search</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>GA4未命中</t>
+          <t>GA4已命中</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>GA4未命中：需确认 seeed.cc / 中文站是否接入当前 GA4 Property，或下一次用 /solutions 过滤专项拉数</t>
+          <t>有流量但转化偏弱：优先检查CTA、表单入口和案例承接</t>
         </is>
       </c>
       <c r="P7" t="inlineStr">
@@ -1008,47 +1008,47 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>100.00%</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>待接入 CTA 点击事件</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
           <t>0</t>
         </is>
       </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="I8" t="inlineStr">
-        <is>
-          <t>0.00</t>
-        </is>
-      </c>
-      <c r="J8" t="inlineStr">
-        <is>
-          <t>0.00%</t>
-        </is>
-      </c>
-      <c r="K8" t="inlineStr">
-        <is>
-          <t>待接入 CTA 点击事件</t>
-        </is>
-      </c>
-      <c r="L8" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>未命中</t>
+          <t>Unassigned</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>GA4未命中</t>
+          <t>GA4已命中</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>GA4未命中：需确认 seeed.cc / 中文站是否接入当前 GA4 Property，或下一次用 /solutions 过滤专项拉数</t>
+          <t>样本偏少：先确认埋点和入口曝光，再判断增长</t>
         </is>
       </c>
       <c r="P8" t="inlineStr">
@@ -1095,47 +1095,47 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>4.40</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>100.00%</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>待接入 CTA 点击事件</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
           <t>0</t>
         </is>
       </c>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="I9" t="inlineStr">
-        <is>
-          <t>0.00</t>
-        </is>
-      </c>
-      <c r="J9" t="inlineStr">
-        <is>
-          <t>0.00%</t>
-        </is>
-      </c>
-      <c r="K9" t="inlineStr">
-        <is>
-          <t>待接入 CTA 点击事件</t>
-        </is>
-      </c>
-      <c r="L9" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>未命中</t>
+          <t>Direct</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
         <is>
-          <t>GA4未命中</t>
+          <t>GA4已命中</t>
         </is>
       </c>
       <c r="O9" t="inlineStr">
         <is>
-          <t>GA4未命中：需确认 seeed.cc / 中文站是否接入当前 GA4 Property，或下一次用 /solutions 过滤专项拉数</t>
+          <t>样本偏少：先确认埋点和入口曝光，再判断增长</t>
         </is>
       </c>
       <c r="P9" t="inlineStr">
@@ -1182,47 +1182,47 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
+          <t>26</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>96.33</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>100.00%</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>待接入 CTA 点击事件</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
           <t>0</t>
         </is>
       </c>
-      <c r="H10" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="I10" t="inlineStr">
-        <is>
-          <t>0.00</t>
-        </is>
-      </c>
-      <c r="J10" t="inlineStr">
-        <is>
-          <t>0.00%</t>
-        </is>
-      </c>
-      <c r="K10" t="inlineStr">
-        <is>
-          <t>待接入 CTA 点击事件</t>
-        </is>
-      </c>
-      <c r="L10" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>未命中</t>
+          <t>Direct</t>
         </is>
       </c>
       <c r="N10" t="inlineStr">
         <is>
-          <t>GA4未命中</t>
+          <t>GA4已命中</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>GA4未命中：需确认 seeed.cc / 中文站是否接入当前 GA4 Property，或下一次用 /solutions 过滤专项拉数</t>
+          <t>样本偏少：先确认埋点和入口曝光，再判断增长</t>
         </is>
       </c>
       <c r="P10" t="inlineStr">
@@ -1269,47 +1269,47 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
+          <t>26</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>24.80</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>100.00%</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>待接入 CTA 点击事件</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
           <t>0</t>
         </is>
       </c>
-      <c r="H11" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="I11" t="inlineStr">
-        <is>
-          <t>0.00</t>
-        </is>
-      </c>
-      <c r="J11" t="inlineStr">
-        <is>
-          <t>0.00%</t>
-        </is>
-      </c>
-      <c r="K11" t="inlineStr">
-        <is>
-          <t>待接入 CTA 点击事件</t>
-        </is>
-      </c>
-      <c r="L11" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>未命中</t>
+          <t>Organic Search</t>
         </is>
       </c>
       <c r="N11" t="inlineStr">
         <is>
-          <t>GA4未命中</t>
+          <t>GA4已命中</t>
         </is>
       </c>
       <c r="O11" t="inlineStr">
         <is>
-          <t>GA4未命中：需确认 seeed.cc / 中文站是否接入当前 GA4 Property，或下一次用 /solutions 过滤专项拉数</t>
+          <t>样本偏少：先确认埋点和入口曝光，再判断增长</t>
         </is>
       </c>
       <c r="P11" t="inlineStr">
@@ -1356,47 +1356,47 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
+          <t>65</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>23</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>41.92</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>70.83%</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>待接入 CTA 点击事件</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
           <t>0</t>
         </is>
       </c>
-      <c r="H12" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="I12" t="inlineStr">
-        <is>
-          <t>0.00</t>
-        </is>
-      </c>
-      <c r="J12" t="inlineStr">
-        <is>
-          <t>0.00%</t>
-        </is>
-      </c>
-      <c r="K12" t="inlineStr">
-        <is>
-          <t>待接入 CTA 点击事件</t>
-        </is>
-      </c>
-      <c r="L12" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>未命中</t>
+          <t>Direct</t>
         </is>
       </c>
       <c r="N12" t="inlineStr">
         <is>
-          <t>GA4未命中</t>
+          <t>GA4已命中</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>GA4未命中：需确认 seeed.cc / 中文站是否接入当前 GA4 Property，或下一次用 /solutions 过滤专项拉数</t>
+          <t>样本偏少：先确认埋点和入口曝光，再判断增长</t>
         </is>
       </c>
       <c r="P12" t="inlineStr">
@@ -1443,47 +1443,47 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
+          <t>60</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>27</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>7.24</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>100.00%</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>待接入 CTA 点击事件</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
           <t>0</t>
         </is>
       </c>
-      <c r="H13" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="I13" t="inlineStr">
-        <is>
-          <t>0.00</t>
-        </is>
-      </c>
-      <c r="J13" t="inlineStr">
-        <is>
-          <t>0.00%</t>
-        </is>
-      </c>
-      <c r="K13" t="inlineStr">
-        <is>
-          <t>待接入 CTA 点击事件</t>
-        </is>
-      </c>
-      <c r="L13" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>未命中</t>
+          <t>Direct</t>
         </is>
       </c>
       <c r="N13" t="inlineStr">
         <is>
-          <t>GA4未命中</t>
+          <t>GA4已命中</t>
         </is>
       </c>
       <c r="O13" t="inlineStr">
         <is>
-          <t>GA4未命中：需确认 seeed.cc / 中文站是否接入当前 GA4 Property，或下一次用 /solutions 过滤专项拉数</t>
+          <t>样本偏少：先确认埋点和入口曝光，再判断增长</t>
         </is>
       </c>
       <c r="P13" t="inlineStr">
@@ -1589,37 +1589,37 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>389765</t>
+          <t>367730</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>406278</t>
+          <t>382800</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>910049</t>
+          <t>845154</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>15286</t>
+          <t>14733</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>3.76%</t>
+          <t>3.85%</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>12.23%</t>
+          <t>12.54%</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>21.97</t>
+          <t>21.58</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
@@ -1656,37 +1656,37 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>296145</t>
+          <t>279666</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>321421</t>
+          <t>303587</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>756231</t>
+          <t>700379</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>18525</t>
+          <t>18288</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>5.76%</t>
+          <t>6.02%</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>16.06%</t>
+          <t>16.70%</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>36.56</t>
+          <t>36.71</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
@@ -1723,37 +1723,37 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>126008</t>
+          <t>121648</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>136468</t>
+          <t>131771</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>261949</t>
+          <t>249623</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>6066</t>
+          <t>5960</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>4.44%</t>
+          <t>4.52%</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>43.63%</t>
+          <t>43.25%</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>40.21</t>
+          <t>40.61</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
@@ -1790,37 +1790,37 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>93622</t>
+          <t>90316</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>103163</t>
+          <t>99590</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>259047</t>
+          <t>248116</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>7214</t>
+          <t>7175</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>6.99%</t>
+          <t>7.20%</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>9.28%</t>
+          <t>9.44%</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>39.15</t>
+          <t>39.31</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
@@ -1857,37 +1857,37 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>83105</t>
+          <t>77117</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>89689</t>
+          <t>83278</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>233812</t>
+          <t>212557</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>5493</t>
+          <t>5407</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>6.12%</t>
+          <t>6.49%</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>6.62%</t>
+          <t>6.82%</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>42.03</t>
+          <t>42.02</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
@@ -2013,42 +2013,42 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>175205</t>
+          <t>107827</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>81525</t>
+          <t>60284</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>89446</t>
+          <t>66679</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>84.07%</t>
+          <t>81.21%</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>15.93%</t>
+          <t>18.79%</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>27.45</t>
+          <t>28.93</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>2707</t>
+          <t>2639</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>2707</t>
+          <t>2639</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
@@ -2090,42 +2090,42 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>64270</t>
+          <t>59190</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>24088</t>
+          <t>22462</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>25459</t>
+          <t>23712</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>85.74%</t>
+          <t>86.50%</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>14.26%</t>
+          <t>13.50%</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>24.47</t>
+          <t>25.25</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>1099</t>
+          <t>1015</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>1099</t>
+          <t>1015</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
@@ -2167,42 +2167,42 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>63655</t>
+          <t>57825</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>16922</t>
+          <t>15472</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>18203</t>
+          <t>16673</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>90.23%</t>
+          <t>90.30%</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>9.77%</t>
+          <t>9.70%</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>57.31</t>
+          <t>57.09</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>1140</t>
+          <t>1056</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>1140</t>
+          <t>1056</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
@@ -2234,52 +2234,52 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>/reTerminal-E1002-p-6533.html</t>
+          <t>/XIAO-nRF52840-Wio-SX1262-Kit-for-Meshtastic-p-6400.html</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>reTerminal E1002 | E Ink Spectra 6 Full Color ESP32-S3 ePaper Display with 3-Month Battery Life</t>
+          <t>Meshtastic Development Kit</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>60415</t>
+          <t>39503</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>19067</t>
+          <t>14394</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>20000</t>
+          <t>15339</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>87.55%</t>
+          <t>86.88%</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>12.45%</t>
+          <t>13.12%</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>21.80</t>
+          <t>28.04</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>414</t>
+          <t>822</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>414</t>
+          <t>822</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
@@ -2289,7 +2289,7 @@
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>转化处于可优化区间，建议做渠道和页面拆解</t>
+          <t>转化表现较强，可继续放大有效渠道</t>
         </is>
       </c>
       <c r="O5" t="inlineStr">
@@ -2311,52 +2311,52 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>/XIAO-nRF52840-Wio-SX1262-Kit-for-Meshtastic-p-6400.html</t>
+          <t>/Wio-Tracker-L1-Pro-p-6454.html</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Meshtastic Development Kit</t>
+          <t>Meshtastic Device/ Rugged Meshtastic Device with Battery, OLED &amp; GPS from Seeed Studio.</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>39752</t>
+          <t>33585</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>14462</t>
+          <t>12045</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>15415</t>
+          <t>13141</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>86.94%</t>
+          <t>87.25%</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>13.06%</t>
+          <t>12.75%</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>28.06</t>
+          <t>33.50</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>826</t>
+          <t>715</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>826</t>
+          <t>715</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
@@ -2388,52 +2388,52 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>/Wio-Tracker-L1-Pro-p-6454.html</t>
+          <t>/SenseCAP-Solar-Node-P1-Pro-for-Meshtastic-LoRa-p-6412.html</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Meshtastic Device/ Rugged Meshtastic Device with Battery, OLED &amp; GPS from Seeed Studio.</t>
+          <t>Meshtastic Solar Powered Node / Repeater with built-in GPS and Battery</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>34776</t>
+          <t>33326</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>12444</t>
+          <t>12415</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>13587</t>
+          <t>13521</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>86.22%</t>
+          <t>83.93%</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>13.78%</t>
+          <t>16.07%</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>32.90</t>
+          <t>41.78</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>741</t>
+          <t>574</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>741</t>
+          <t>574</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
@@ -2443,7 +2443,7 @@
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>转化表现较强，可继续放大有效渠道</t>
+          <t>转化处于可优化区间，建议做渠道和页面拆解</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
@@ -2465,52 +2465,52 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>/SenseCAP-Solar-Node-P1-Pro-for-Meshtastic-LoRa-p-6412.html</t>
+          <t>/XIAO-ESP32S3-Sense-p-5639.html</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Meshtastic Solar Powered Node / Repeater with built-in GPS and Battery</t>
+          <t>Mini ESP-CAM Dev Board for Edge AI - XIAO ESP32S3 Sense</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>33696</t>
+          <t>32571</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>12511</t>
+          <t>12489</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>13626</t>
+          <t>13772</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>84.04%</t>
+          <t>81.92%</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>15.96%</t>
+          <t>18.08%</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>41.59</t>
+          <t>34.38</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>581</t>
+          <t>659</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>581</t>
+          <t>659</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
@@ -2542,52 +2542,52 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>/reTerminal-E1001-p-6534.html</t>
+          <t>/reTerminal-E1002-p-6533.html</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>reTerminal E1001 | Always-on ESP32-S3 ePaper Display with 3-Month Battery Life</t>
+          <t>reTerminal E1002 | E Ink Spectra 6 Full Color ESP32-S3 ePaper Display with 3-Month Battery Life</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>33463</t>
+          <t>32392</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>12154</t>
+          <t>11214</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>12883</t>
+          <t>11855</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>74.75%</t>
+          <t>80.21%</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>25.25%</t>
+          <t>19.79%</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>27.36</t>
+          <t>26.18</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>495</t>
+          <t>319</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>495</t>
+          <t>319</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
@@ -2619,52 +2619,52 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>/XIAO-ESP32S3-Sense-p-5639.html</t>
+          <t>/reTerminal-E1001-p-6534.html</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Mini ESP-CAM Dev Board for Edge AI - XIAO ESP32S3 Sense</t>
+          <t>reTerminal E1001 | Always-on ESP32-S3 ePaper Display with 3-Month Battery Life</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>32571</t>
+          <t>31237</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>12489</t>
+          <t>11517</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>13772</t>
+          <t>12194</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>81.92%</t>
+          <t>73.42%</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>18.08%</t>
+          <t>26.58%</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>34.38</t>
+          <t>27.95</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>659</t>
+          <t>446</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>659</t>
+          <t>446</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
@@ -2850,42 +2850,42 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>/catalogsearch/result/</t>
+          <t>/customer_order_shipment.html</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Search results for: ''</t>
+          <t>Track Shipment</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>27015</t>
+          <t>26483</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>9271</t>
+          <t>10211</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>9968</t>
+          <t>13181</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>86.64%</t>
+          <t>78.94%</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>13.36%</t>
+          <t>21.06%</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>53.21</t>
+          <t>12.46</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
@@ -2900,7 +2900,7 @@
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>其他</t>
+          <t>产品页</t>
         </is>
       </c>
       <c r="N13" t="inlineStr">
@@ -2927,52 +2927,52 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>/customer_order_shipment.html</t>
+          <t>/respeaker-clip-wearable-ai-recorder.html</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Track Shipment</t>
+          <t>reSpeaker Clip: Open Wearable AI Recorder | Voice AI Agent | AI Note Taker</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>26527</t>
+          <t>23567</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>10226</t>
+          <t>8791</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>13203</t>
+          <t>9484</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>78.96%</t>
+          <t>88.35%</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>21.04%</t>
+          <t>11.65%</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>12.46</t>
+          <t>34.95</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>387</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>387</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
@@ -2982,7 +2982,7 @@
       </c>
       <c r="N14" t="inlineStr">
         <is>
-          <t>转化偏弱，需检查表单、咨询入口和购买链路</t>
+          <t>转化处于可优化区间，建议做渠道和页面拆解</t>
         </is>
       </c>
       <c r="O14" t="inlineStr">
@@ -3004,62 +3004,62 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>/reTerminal-E1004-p-6692.html</t>
+          <t>/sales/order/history/</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>reTerminal E1004 13.3" Full-color ePaper Display</t>
+          <t>My Orders</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>25882</t>
+          <t>23251</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>10289</t>
+          <t>8043</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>10844</t>
+          <t>9398</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>89.13%</t>
+          <t>88.66%</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>10.87%</t>
+          <t>11.34%</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>24.27</t>
+          <t>26.25</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>237</t>
+          <t>20</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>237</t>
+          <t>20</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>产品页</t>
+          <t>其他</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>转化处于可优化区间，建议做渠道和页面拆解</t>
+          <t>转化偏弱，需检查表单、咨询入口和购买链路</t>
         </is>
       </c>
       <c r="O15" t="inlineStr">
@@ -3081,52 +3081,52 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>/respeaker-clip-wearable-ai-recorder.html</t>
+          <t>/Home-Assistant-Green-p-5792.html</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>reSpeaker Clip: Open Wearable AI Recorder | Voice AI Agent | AI Note Taker</t>
+          <t>Home Assistant Green - Seeed Studio</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>24161</t>
+          <t>22181</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>8975</t>
+          <t>8400</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>9672</t>
+          <t>8872</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>88.54%</t>
+          <t>79.81%</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>11.46%</t>
+          <t>20.19%</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>34.73</t>
+          <t>22.12</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>393</t>
+          <t>564</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>393</t>
+          <t>564</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
@@ -3136,7 +3136,7 @@
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>转化处于可优化区间，建议做渠道和页面拆解</t>
+          <t>转化表现较强，可继续放大有效渠道</t>
         </is>
       </c>
       <c r="O16" t="inlineStr">
@@ -3158,52 +3158,52 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>/sales/order/history/</t>
+          <t>/eu_warehouse</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>My Orders</t>
+          <t>EU_Warehouse</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>23540</t>
+          <t>22116</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>8148</t>
+          <t>9293</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>9523</t>
+          <t>9930</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>88.62%</t>
+          <t>84.96%</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>11.38%</t>
+          <t>15.04%</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>26.23</t>
+          <t>41.72</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>0</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>0</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
@@ -3235,62 +3235,62 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>/eu_warehouse</t>
+          <t>/Seeed-Studio-XIAO-ESP32C6-p-5884.html</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>EU_Warehouse</t>
+          <t>Tiny Matter-Native Board for Smart Home - XIAO ESP32C6</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>22994</t>
+          <t>21624</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>9652</t>
+          <t>8163</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>10304</t>
+          <t>8905</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>85.03%</t>
+          <t>83.92%</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>14.97%</t>
+          <t>16.08%</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>41.72</t>
+          <t>30.73</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>218</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>218</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>其他</t>
+          <t>产品页</t>
         </is>
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>转化偏弱，需检查表单、咨询入口和购买链路</t>
+          <t>转化处于可优化区间，建议做渠道和页面拆解</t>
         </is>
       </c>
       <c r="O18" t="inlineStr">
@@ -3312,52 +3312,52 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>/Home-Assistant-Green-p-5792.html</t>
+          <t>/Grove-2-5A-DC-Current-Sensor-ACS70331-p-2929.html</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Home Assistant Green - Seeed Studio</t>
+          <t>Grove - 2.5A DC Current Sensor(ACS70331) - Seeed Studio</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>22625</t>
+          <t>20986</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>8596</t>
+          <t>10950</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>9085</t>
+          <t>10948</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>79.63%</t>
+          <t>88.32%</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>20.37%</t>
+          <t>11.68%</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>22.29</t>
+          <t>1.43</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>572</t>
+          <t>0</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>572</t>
+          <t>0</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
@@ -3367,7 +3367,7 @@
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>转化表现较强，可继续放大有效渠道</t>
+          <t>转化偏弱，需检查表单、咨询入口和购买链路</t>
         </is>
       </c>
       <c r="O19" t="inlineStr">
@@ -3389,57 +3389,57 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>/Seeed-Studio-XIAO-ESP32C6-p-5884.html</t>
+          <t>/checkout/cart/</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Tiny Matter-Native Board for Smart Home - XIAO ESP32C6</t>
+          <t>Seeed Studio Bazaar, The IoT Hardware enabler.</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>21624</t>
+          <t>20631</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>8163</t>
+          <t>5162</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>8905</t>
+          <t>5403</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>83.92%</t>
+          <t>93.41%</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>16.08%</t>
+          <t>6.59%</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>30.73</t>
+          <t>15.28</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>218</t>
+          <t>57</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>218</t>
+          <t>57</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>产品页</t>
+          <t>购买/购物车</t>
         </is>
       </c>
       <c r="N20" t="inlineStr">
@@ -3466,52 +3466,52 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>/Meshtastic-Starter-Kit-Ready-to-Use-Off-Grid-Instant-Reliable-Communication.html</t>
+          <t>/Wio-SX1262-with-XIAO-ESP32S3-p-5982.html</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Meshtastic Starter Kit, Off-Grid Network without Cell Service, Plug-and-Play</t>
+          <t>XIAO ESP32S3 &amp; Wio-SX1262 Kit for Meshtastic &amp; LoRa</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>21363</t>
+          <t>20512</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>8777</t>
+          <t>7620</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>9314</t>
+          <t>8297</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>90.87%</t>
+          <t>81.60%</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>9.13%</t>
+          <t>18.40%</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>34.25</t>
+          <t>42.04</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>399</t>
+          <t>409</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>399</t>
+          <t>409</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
@@ -3543,52 +3543,52 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>/checkout/cart/</t>
+          <t>/expresscheckout.html</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Seeed Studio Bazaar, The IoT Hardware enabler.</t>
+          <t>Express Checkout</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>21161</t>
+          <t>19828</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>5285</t>
+          <t>6773</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>5539</t>
+          <t>7337</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>93.55%</t>
+          <t>91.82%</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>6.45%</t>
+          <t>8.18%</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>15.31</t>
+          <t>136.61</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>57</t>
+          <t>9024</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>57</t>
+          <t>9024</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
@@ -3598,7 +3598,7 @@
       </c>
       <c r="N22" t="inlineStr">
         <is>
-          <t>转化处于可优化区间，建议做渠道和页面拆解</t>
+          <t>转化表现较强，可继续放大有效渠道</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
@@ -3620,52 +3620,52 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>/Grove-2-5A-DC-Current-Sensor-ACS70331-p-2929.html</t>
+          <t>/reTerminal-E1004-p-6692.html</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Grove - 2.5A DC Current Sensor(ACS70331) - Seeed Studio</t>
+          <t>reTerminal E1004 13.3" Full-color ePaper Display</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>20986</t>
+          <t>19425</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>10950</t>
+          <t>7542</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>10948</t>
+          <t>8048</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>88.32%</t>
+          <t>85.98%</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>11.68%</t>
+          <t>14.02%</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>1.43</t>
+          <t>29.02</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>221</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>221</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
@@ -3675,7 +3675,7 @@
       </c>
       <c r="N23" t="inlineStr">
         <is>
-          <t>转化偏弱，需检查表单、咨询入口和购买链路</t>
+          <t>转化处于可优化区间，建议做渠道和页面拆解</t>
         </is>
       </c>
       <c r="O23" t="inlineStr">
@@ -3697,52 +3697,52 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>/Wio-SX1262-with-XIAO-ESP32S3-p-5982.html</t>
+          <t>/Meshtastic-Starter-Kit-Ready-to-Use-Off-Grid-Instant-Reliable-Communication.html</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>XIAO ESP32S3 &amp; Wio-SX1262 Kit for Meshtastic &amp; LoRa</t>
+          <t>Meshtastic Starter Kit, Off-Grid Network without Cell Service, Plug-and-Play</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>20634</t>
+          <t>18976</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>7653</t>
+          <t>7457</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>8331</t>
+          <t>7914</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>81.65%</t>
+          <t>89.41%</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>18.35%</t>
+          <t>10.59%</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>42.13</t>
+          <t>37.58</t>
         </is>
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>414</t>
+          <t>347</t>
         </is>
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>414</t>
+          <t>347</t>
         </is>
       </c>
       <c r="M24" t="inlineStr">
@@ -3774,62 +3774,62 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>/expresscheckout.html</t>
+          <t>/reBot-Arm-B601-RS-Assembled-Kit-with-Gripper-p-6865.html</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Express Checkout</t>
+          <t>reBot Arm B601-RS : a low-cost 6-degree-of-freedom open-source robotic arm built based on the Lingzu Robstride series motors</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>19947</t>
+          <t>18570</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>6809</t>
+          <t>5882</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>7375</t>
+          <t>6221</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>91.76%</t>
+          <t>85.00%</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>8.24%</t>
+          <t>15.00%</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>136.49</t>
+          <t>25.18</t>
         </is>
       </c>
       <c r="K25" t="inlineStr">
         <is>
-          <t>9080</t>
+          <t>136</t>
         </is>
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>9080</t>
+          <t>136</t>
         </is>
       </c>
       <c r="M25" t="inlineStr">
         <is>
-          <t>购买/购物车</t>
+          <t>产品页</t>
         </is>
       </c>
       <c r="N25" t="inlineStr">
         <is>
-          <t>转化表现较强，可继续放大有效渠道</t>
+          <t>转化处于可优化区间，建议做渠道和页面拆解</t>
         </is>
       </c>
       <c r="O25" t="inlineStr">
@@ -3851,52 +3851,52 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>/reBot-Arm-B601-RS-Assembled-Kit-with-Gripper-p-6865.html</t>
+          <t>/Grove-5A-DC-AC-Current-Sensor-ACS70331-p-2928.html</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>reBot Arm B601-RS : a low-cost 6-degree-of-freedom open-source robotic arm built based on the Lingzu Robstride series motors</t>
+          <t>Grove - ±5A DC/AC Current Sensor (ACS70331) - Seeed Studio</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>19035</t>
+          <t>18276</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>6020</t>
+          <t>9737</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>6365</t>
+          <t>9735</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>85.28%</t>
+          <t>88.50%</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>14.72%</t>
+          <t>11.50%</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>24.98</t>
+          <t>1.32</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t>137</t>
+          <t>0</t>
         </is>
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>137</t>
+          <t>0</t>
         </is>
       </c>
       <c r="M26" t="inlineStr">
@@ -3906,7 +3906,7 @@
       </c>
       <c r="N26" t="inlineStr">
         <is>
-          <t>转化处于可优化区间，建议做渠道和页面拆解</t>
+          <t>转化偏弱，需检查表单、咨询入口和购买链路</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
@@ -3928,52 +3928,52 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>/Grove-5A-DC-AC-Current-Sensor-ACS70331-p-2928.html</t>
+          <t>/Minichord-Synthesizer-p-6414.html</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Grove - ±5A DC/AC Current Sensor (ACS70331) - Seeed Studio</t>
+          <t>Minichord Synthesizer - Innovative Open-Source MIDI Musical Synthesizer Device</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>18276</t>
+          <t>18032</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>9737</t>
+          <t>5561</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>9735</t>
+          <t>6046</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>88.50%</t>
+          <t>83.97%</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>11.50%</t>
+          <t>16.03%</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>1.32</t>
+          <t>14.15</t>
         </is>
       </c>
       <c r="K27" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>301</t>
         </is>
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>301</t>
         </is>
       </c>
       <c r="M27" t="inlineStr">
@@ -3983,7 +3983,7 @@
       </c>
       <c r="N27" t="inlineStr">
         <is>
-          <t>转化偏弱，需检查表单、咨询入口和购买链路</t>
+          <t>转化处于可优化区间，建议做渠道和页面拆解</t>
         </is>
       </c>
       <c r="O27" t="inlineStr">
@@ -4005,52 +4005,52 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>/reCamera-Pro-2GB.html</t>
+          <t>/TRMNL-7-5-Inch-OG-DIY-Kit-p-6481.html</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Edge AI Camera with Local AI Inference Seeed Studio</t>
+          <t>TRMNL 7.5" DIY E-ink Dashboard Kit | Seeed Studio x TRMNL Official</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>18196</t>
+          <t>17485</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>7011</t>
+          <t>6527</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>7539</t>
+          <t>7117</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>82.29%</t>
+          <t>85.05%</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>17.71%</t>
+          <t>14.95%</t>
         </is>
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>42.61</t>
+          <t>34.88</t>
         </is>
       </c>
       <c r="K28" t="inlineStr">
         <is>
-          <t>78</t>
+          <t>356</t>
         </is>
       </c>
       <c r="L28" t="inlineStr">
         <is>
-          <t>78</t>
+          <t>356</t>
         </is>
       </c>
       <c r="M28" t="inlineStr">
@@ -4060,7 +4060,7 @@
       </c>
       <c r="N28" t="inlineStr">
         <is>
-          <t>转化处于可优化区间，建议做渠道和页面拆解</t>
+          <t>转化表现较强，可继续放大有效渠道</t>
         </is>
       </c>
       <c r="O28" t="inlineStr">
@@ -4082,62 +4082,62 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>/Minichord-Synthesizer-p-6414.html</t>
+          <t>/customer/account/login/referer/aHR0cHM6Ly93d3cuc2VlZWRzdHVkaW8uY29tL2NoZWNrb3V0L2NhcnQvY2hlY2tvdXQv/</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Minichord Synthesizer - Innovative Open-Source MIDI Musical Synthesizer Device</t>
+          <t>Customer Login</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>18110</t>
+          <t>17213</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>5577</t>
+          <t>7372</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>6062</t>
+          <t>7470</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>84.02%</t>
+          <t>93.33%</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>15.98%</t>
+          <t>6.67%</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>14.19</t>
+          <t>15.40</t>
         </is>
       </c>
       <c r="K29" t="inlineStr">
         <is>
-          <t>305</t>
+          <t>0</t>
         </is>
       </c>
       <c r="L29" t="inlineStr">
         <is>
-          <t>305</t>
+          <t>0</t>
         </is>
       </c>
       <c r="M29" t="inlineStr">
         <is>
-          <t>产品页</t>
+          <t>其他</t>
         </is>
       </c>
       <c r="N29" t="inlineStr">
         <is>
-          <t>转化表现较强，可继续放大有效渠道</t>
+          <t>转化偏弱，需检查表单、咨询入口和购买链路</t>
         </is>
       </c>
       <c r="O29" t="inlineStr">
@@ -4159,62 +4159,62 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>/checkout/cart</t>
+          <t>/ReSpeaker-XVF3800-USB-Mic-Array-p-6488.html</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Seeed Studio Bazaar, The IoT Hardware enabler.</t>
+          <t>reSpeaker USB 4-Microphone Array: AI-Powered XMOS XVF3800|Seeed Studio</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>17650</t>
+          <t>16709</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>5021</t>
+          <t>6661</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>5454</t>
+          <t>6961</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>94.43%</t>
+          <t>72.52%</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>5.57%</t>
+          <t>27.48%</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>33.98</t>
+          <t>16.68</t>
         </is>
       </c>
       <c r="K30" t="inlineStr">
         <is>
-          <t>53</t>
+          <t>102</t>
         </is>
       </c>
       <c r="L30" t="inlineStr">
         <is>
-          <t>53</t>
+          <t>102</t>
         </is>
       </c>
       <c r="M30" t="inlineStr">
         <is>
-          <t>购买/购物车</t>
+          <t>产品页</t>
         </is>
       </c>
       <c r="N30" t="inlineStr">
         <is>
-          <t>转化偏弱，需检查表单、咨询入口和购买链路</t>
+          <t>转化处于可优化区间，建议做渠道和页面拆解</t>
         </is>
       </c>
       <c r="O30" t="inlineStr">
@@ -4236,52 +4236,52 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>/reTerminal-E1003-p-6731.html</t>
+          <t>/Seeed-Studio-XIAO-ESP32C5-p-6609.html</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>reTerminal E1003 10.3” Touch ePaper Dashboard Display | Fast Refresh, 16-Level Grayscale</t>
+          <t>XIAO ESP32-C5 Dual-band 2.4/5 GHz Wi‑Fi MCU for IoT Devices</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>17572</t>
+          <t>16674</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>7489</t>
+          <t>6033</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>7875</t>
+          <t>6490</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>87.50%</t>
+          <t>84.55%</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>12.50%</t>
+          <t>15.45%</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>20.55</t>
+          <t>30.74</t>
         </is>
       </c>
       <c r="K31" t="inlineStr">
         <is>
-          <t>207</t>
+          <t>427</t>
         </is>
       </c>
       <c r="L31" t="inlineStr">
         <is>
-          <t>207</t>
+          <t>427</t>
         </is>
       </c>
       <c r="M31" t="inlineStr">
@@ -4291,7 +4291,7 @@
       </c>
       <c r="N31" t="inlineStr">
         <is>
-          <t>转化处于可优化区间，建议做渠道和页面拆解</t>
+          <t>转化表现较强，可继续放大有效渠道</t>
         </is>
       </c>
       <c r="O31" t="inlineStr">
@@ -4392,7 +4392,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>1161048</t>
+          <t>1087293</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -4402,7 +4402,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>最近14天 vs 前14天: 上升1.6%</t>
+          <t>最近14天 vs 前14天: 上升4.4%</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -4427,7 +4427,7 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>2026-07-28T08:17:59</t>
+          <t>2026-07-28T08:59:07</t>
         </is>
       </c>
     </row>
@@ -4454,7 +4454,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>1240383</t>
+          <t>1162076</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -4464,7 +4464,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>最近14天 vs 前14天: 上升1.4%</t>
+          <t>最近14天 vs 前14天: 上升4.2%</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -4489,7 +4489,7 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>2026-07-28T08:17:59</t>
+          <t>2026-07-28T08:59:07</t>
         </is>
       </c>
     </row>
@@ -4551,7 +4551,7 @@
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>2026-07-28T08:17:59</t>
+          <t>2026-07-28T08:59:07</t>
         </is>
       </c>
     </row>
@@ -4578,7 +4578,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>31.90</t>
+          <t>32.09</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -4588,7 +4588,7 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>最近14天 vs 前14天: 下降4.2%</t>
+          <t>最近14天 vs 前14天: 下降4.4%</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -4613,7 +4613,7 @@
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>2026-07-28T08:17:59</t>
+          <t>2026-07-28T08:59:07</t>
         </is>
       </c>
     </row>
@@ -4640,7 +4640,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>15.62%</t>
+          <t>16.14%</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -4650,7 +4650,7 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>最近14天 vs 前14天: 上升71.8%</t>
+          <t>最近14天 vs 前14天: 上升67.7%</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -4675,7 +4675,7 @@
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>2026-07-28T08:17:59</t>
+          <t>2026-07-28T08:59:07</t>
         </is>
       </c>
     </row>
@@ -4737,7 +4737,7 @@
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>2026-07-28T08:17:59</t>
+          <t>2026-07-28T08:59:07</t>
         </is>
       </c>
     </row>
@@ -4764,7 +4764,7 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>/ / /SenseCAP-Card-Tracker-T1000-E-for-Meshtastic-p-5913.html / /checkout/cart/ / /reTerminal-E1002-p-6533.html / /XIAO-nRF52840-Wio-SX1262-Kit-for-Meshtastic-p-6400.html</t>
+          <t>/ / /SenseCAP-Card-Tracker-T1000-E-for-Meshtastic-p-5913.html / /checkout/cart/ / /XIAO-nRF52840-Wio-SX1262-Kit-for-Meshtastic-p-6400.html / /Wio-Tracker-L1-Pro-p-6454.html</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -4799,7 +4799,7 @@
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>2026-07-28T08:17:59</t>
+          <t>2026-07-28T08:59:07</t>
         </is>
       </c>
     </row>
@@ -4826,7 +4826,7 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>61215</t>
+          <t>59943</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -4836,7 +4836,7 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>最近14天 vs 前14天: 上升11.3%</t>
+          <t>最近14天 vs 前14天: 上升10.2%</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
@@ -4861,7 +4861,7 @@
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>2026-07-28T08:17:59</t>
+          <t>2026-07-28T08:59:07</t>
         </is>
       </c>
     </row>
@@ -4888,7 +4888,7 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>4.94%</t>
+          <t>5.16%</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -4898,7 +4898,7 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>最近14天 vs 前14天: 上升9.8%</t>
+          <t>最近14天 vs 前14天: 上升5.7%</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
@@ -4908,7 +4908,7 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>转化处于可优化区间，建议做渠道和页面拆解</t>
+          <t>转化表现较强，可继续放大有效渠道</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
@@ -4923,7 +4923,7 @@
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>2026-07-28T08:17:59</t>
+          <t>2026-07-28T08:59:07</t>
         </is>
       </c>
     </row>
@@ -4985,7 +4985,7 @@
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>2026-07-28T08:17:59</t>
+          <t>2026-07-28T08:59:07</t>
         </is>
       </c>
     </row>
@@ -5136,22 +5136,22 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>14663</t>
+          <t>12852</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>13946</t>
+          <t>12164</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>573</t>
+          <t>535</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>3.91%</t>
+          <t>4.16%</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">

</xml_diff>

<commit_message>
Scope Feishu tables to solution pages
</commit_message>
<xml_diff>
--- a/exports/feishu-base-import/seeed_解决方案增长_多维表格导入.xlsx
+++ b/exports/feishu-base-import/seeed_解决方案增长_多维表格导入.xlsx
@@ -5,7 +5,7 @@
     <sheet name="01_方案增长总览表" sheetId="1" r:id="rId1"/>
     <sheet name="02_转化漏斗表" sheetId="2" r:id="rId2"/>
     <sheet name="03_流量来源渠道" sheetId="3" r:id="rId3"/>
-    <sheet name="04_热门页面与行为" sheetId="4" r:id="rId4"/>
+    <sheet name="04_解决方案页面与行为" sheetId="4" r:id="rId4"/>
     <sheet name="05_社媒平台表现" sheetId="5" r:id="rId5"/>
   </sheets>
 </workbook>
@@ -84,7 +84,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>8338</t>
+          <t>83</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -104,7 +104,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>校园安全管理</t>
+          <t>智能仓储管理</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
@@ -190,7 +190,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>3696</t>
+          <t>0</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -200,7 +200,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>58</t>
+          <t>0</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -294,7 +294,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>18</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -346,7 +346,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>361</t>
+          <t>0</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -356,7 +356,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -398,7 +398,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>4164</t>
+          <t>0</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -408,7 +408,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>109</t>
+          <t>0</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -450,7 +450,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>64</t>
+          <t>0</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -658,7 +658,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>0</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -710,7 +710,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>0</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -893,37 +893,37 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>97033</t>
+          <t>20</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>100757</t>
+          <t>20</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>226449</t>
+          <t>33</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>3788</t>
+          <t>0</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>3.76%</t>
+          <t>0.00%</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>9.15%</t>
+          <t>20.00%</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>21.82</t>
+          <t>26.10</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
@@ -933,7 +933,7 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>转化处于可优化区间，建议做渠道和页面拆解</t>
+          <t>转化偏弱，需检查表单、咨询入口和购买链路</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
@@ -960,37 +960,37 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>67380</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>73144</t>
+          <t>11</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>173271</t>
+          <t>20</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>4774</t>
+          <t>0</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>6.53%</t>
+          <t>0.00%</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>12.28%</t>
+          <t>9.09%</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>39.47</t>
+          <t>14.27</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
@@ -1000,7 +1000,7 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>转化表现较强，可继续放大有效渠道</t>
+          <t>转化偏弱，需检查表单、咨询入口和购买链路</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
@@ -1022,42 +1022,42 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Paid Search</t>
+          <t>Referral</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>21841</t>
+          <t>5</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>23540</t>
+          <t>6</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>59146</t>
+          <t>15</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>1525</t>
+          <t>0</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>6.48%</t>
+          <t>0.00%</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>5.97%</t>
+          <t>0.00%</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>43.00</t>
+          <t>15.16</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
@@ -1067,7 +1067,7 @@
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>转化表现较强，可继续放大有效渠道</t>
+          <t>转化偏弱，需检查表单、咨询入口和购买链路</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
@@ -1089,42 +1089,42 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Referral</t>
+          <t>Paid Search</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>21287</t>
+          <t>2</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>23431</t>
+          <t>2</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>58144</t>
+          <t>6</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>1699</t>
+          <t>0</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>7.25%</t>
+          <t>0.00%</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>7.83%</t>
+          <t>0.00%</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>40.10</t>
+          <t>13.50</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
@@ -1134,7 +1134,7 @@
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>转化表现较强，可继续放大有效渠道</t>
+          <t>转化偏弱，需检查表单、咨询入口和购买链路</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
@@ -1161,37 +1161,37 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>22295</t>
+          <t>2</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>24402</t>
+          <t>2</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>49348</t>
+          <t>4</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>1204</t>
+          <t>0</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>4.93%</t>
+          <t>0.00%</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>27.48%</t>
+          <t>0.00%</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>49.49</t>
+          <t>20.50</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
@@ -1201,7 +1201,7 @@
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>转化处于可优化区间，建议做渠道和页面拆解</t>
+          <t>转化偏弱，需检查表单、咨询入口和购买链路</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
@@ -1307,57 +1307,57 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>/</t>
+          <t>/solutions-by-scenarios</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Seeed Studio Bazaar, The IoT Hardware enabler.</t>
+          <t>Solutions by Scenarios</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>20085</t>
+          <t>57</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>15114</t>
+          <t>28</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>16569</t>
+          <t>29</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>85.50%</t>
+          <t>89.66%</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>14.50%</t>
+          <t>10.34%</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>27.42</t>
+          <t>21.24</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>66</t>
+          <t>0</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>66</t>
+          <t>0</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>首页</t>
+          <t>解决方案</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
@@ -1384,62 +1384,62 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>/SenseCAP-Card-Tracker-T1000-E-for-Meshtastic-p-5913.html</t>
+          <t>/solutions/intelligent-video-analytics</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Meshtastic Device - SenseCAP Card Tracker T1000-E</t>
+          <t>Intelligent Video Analytics - solution</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>15360</t>
+          <t>17</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>5804</t>
+          <t>10</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>6137</t>
+          <t>11</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>89.93%</t>
+          <t>81.82%</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>10.07%</t>
+          <t>18.18%</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>25.04</t>
+          <t>23.45</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>288</t>
+          <t>0</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>288</t>
+          <t>0</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>产品页</t>
+          <t>解决方案</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>转化处于可优化区间，建议做渠道和页面拆解</t>
+          <t>转化偏弱，需检查表单、咨询入口和购买链路</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
@@ -1461,62 +1461,62 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>/checkout/cart/</t>
+          <t>/solutions/smart-warehouse-management</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Shopping Cart</t>
+          <t>404 Page not found</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>13325</t>
+          <t>6</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>3632</t>
+          <t>2</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>3898</t>
+          <t>2</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>95.02%</t>
+          <t>100.00%</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>4.98%</t>
+          <t>0.00%</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>55.05</t>
+          <t>2.50</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>266</t>
+          <t>0</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>266</t>
+          <t>0</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>购买/购物车</t>
+          <t>解决方案</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>转化表现较强，可继续放大有效渠道</t>
+          <t>转化偏弱，需检查表单、咨询入口和购买链路</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
@@ -1538,62 +1538,62 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>/reTerminal-E1001-p-6534.html</t>
+          <t>/solutions-by-scenarios</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>reTerminal E1001 | Always-on ESP32-S3 ePaper Display with 3-Month Battery Life</t>
+          <t>更多场景划分的解决方案</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>10222</t>
+          <t>2</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>3559</t>
+          <t>1</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>3732</t>
+          <t>1</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>80.73%</t>
+          <t>100.00%</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>19.27%</t>
+          <t>0.00%</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>17.55</t>
+          <t>22.00</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>98</t>
+          <t>0</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>98</t>
+          <t>0</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>产品页</t>
+          <t>解决方案</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>转化处于可优化区间，建议做渠道和页面拆解</t>
+          <t>转化偏弱，需检查表单、咨询入口和购买链路</t>
         </is>
       </c>
       <c r="O5" t="inlineStr">
@@ -1615,1220 +1615,65 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>/XIAO-nRF52840-Wio-SX1262-Kit-for-Meshtastic-p-6400.html</t>
+          <t>/solutions/intelligent-video-analytics</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Meshtastic Development Kit</t>
+          <t>インテリジェントビデオ分析 - ソリューション</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>10097</t>
+          <t>1</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>3942</t>
+          <t>1</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>4123</t>
+          <t>2</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>89.81%</t>
+          <t>50.00%</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>10.19%</t>
+          <t>50.00%</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>27.08</t>
+          <t>1.00</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>183</t>
+          <t>0</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>183</t>
+          <t>0</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>产品页</t>
+          <t>解决方案</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>转化处于可优化区间，建议做渠道和页面拆解</t>
+          <t>转化偏弱，需检查表单、咨询入口和购买链路</t>
         </is>
       </c>
       <c r="O6" t="inlineStr">
-        <is>
-          <t>保留高浏览页面；对高跳出或低转化页面优化首屏价值、CTA和内部链接</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>2026-07-20</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>2026-07-26</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>/SenseCAP-Solar-Node-P1-Pro-for-Meshtastic-LoRa-p-6412.html</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>Meshtastic Solar Powered Node / Repeater with built-in GPS and Battery</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>8736</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>2973</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>3220</t>
-        </is>
-      </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>88.98%</t>
-        </is>
-      </c>
-      <c r="I7" t="inlineStr">
-        <is>
-          <t>11.02%</t>
-        </is>
-      </c>
-      <c r="J7" t="inlineStr">
-        <is>
-          <t>45.63</t>
-        </is>
-      </c>
-      <c r="K7" t="inlineStr">
-        <is>
-          <t>156</t>
-        </is>
-      </c>
-      <c r="L7" t="inlineStr">
-        <is>
-          <t>156</t>
-        </is>
-      </c>
-      <c r="M7" t="inlineStr">
-        <is>
-          <t>产品页</t>
-        </is>
-      </c>
-      <c r="N7" t="inlineStr">
-        <is>
-          <t>转化处于可优化区间，建议做渠道和页面拆解</t>
-        </is>
-      </c>
-      <c r="O7" t="inlineStr">
-        <is>
-          <t>保留高浏览页面；对高跳出或低转化页面优化首屏价值、CTA和内部链接</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>2026-07-20</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>2026-07-26</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>/Wio-Tracker-L1-Pro-p-6454.html</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>Meshtastic Device/ Rugged Meshtastic Device with Battery, OLED &amp; GPS from Seeed Studio.</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>8436</t>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>2806</t>
-        </is>
-      </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>3074</t>
-        </is>
-      </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>90.89%</t>
-        </is>
-      </c>
-      <c r="I8" t="inlineStr">
-        <is>
-          <t>9.11%</t>
-        </is>
-      </c>
-      <c r="J8" t="inlineStr">
-        <is>
-          <t>33.99</t>
-        </is>
-      </c>
-      <c r="K8" t="inlineStr">
-        <is>
-          <t>163</t>
-        </is>
-      </c>
-      <c r="L8" t="inlineStr">
-        <is>
-          <t>163</t>
-        </is>
-      </c>
-      <c r="M8" t="inlineStr">
-        <is>
-          <t>产品页</t>
-        </is>
-      </c>
-      <c r="N8" t="inlineStr">
-        <is>
-          <t>转化表现较强，可继续放大有效渠道</t>
-        </is>
-      </c>
-      <c r="O8" t="inlineStr">
-        <is>
-          <t>保留高浏览页面；对高跳出或低转化页面优化首屏价值、CTA和内部链接</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>2026-07-20</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>2026-07-26</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>/reTerminal-E1002-p-6533.html</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>reTerminal E1002 | E Ink Spectra 6 Full Color ESP32-S3 ePaper Display with 3-Month Battery Life</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>8238</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>2638</t>
-        </is>
-      </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>2780</t>
-        </is>
-      </c>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>91.01%</t>
-        </is>
-      </c>
-      <c r="I9" t="inlineStr">
-        <is>
-          <t>8.99%</t>
-        </is>
-      </c>
-      <c r="J9" t="inlineStr">
-        <is>
-          <t>28.17</t>
-        </is>
-      </c>
-      <c r="K9" t="inlineStr">
-        <is>
-          <t>67</t>
-        </is>
-      </c>
-      <c r="L9" t="inlineStr">
-        <is>
-          <t>67</t>
-        </is>
-      </c>
-      <c r="M9" t="inlineStr">
-        <is>
-          <t>产品页</t>
-        </is>
-      </c>
-      <c r="N9" t="inlineStr">
-        <is>
-          <t>转化处于可优化区间，建议做渠道和页面拆解</t>
-        </is>
-      </c>
-      <c r="O9" t="inlineStr">
-        <is>
-          <t>保留高浏览页面；对高跳出或低转化页面优化首屏价值、CTA和内部链接</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>2026-07-20</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>2026-07-26</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>/sensecap-meshtracker-x1-meshtastic-gps-tracker-p-6935.html</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>SenseCAP MeshTracker X1 | Dual-Band Meshtastic GPS Tracker</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>8146</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>2516</t>
-        </is>
-      </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>2738</t>
-        </is>
-      </c>
-      <c r="H10" t="inlineStr">
-        <is>
-          <t>91.20%</t>
-        </is>
-      </c>
-      <c r="I10" t="inlineStr">
-        <is>
-          <t>8.80%</t>
-        </is>
-      </c>
-      <c r="J10" t="inlineStr">
-        <is>
-          <t>45.97</t>
-        </is>
-      </c>
-      <c r="K10" t="inlineStr">
-        <is>
-          <t>237</t>
-        </is>
-      </c>
-      <c r="L10" t="inlineStr">
-        <is>
-          <t>237</t>
-        </is>
-      </c>
-      <c r="M10" t="inlineStr">
-        <is>
-          <t>产品页</t>
-        </is>
-      </c>
-      <c r="N10" t="inlineStr">
-        <is>
-          <t>转化表现较强，可继续放大有效渠道</t>
-        </is>
-      </c>
-      <c r="O10" t="inlineStr">
-        <is>
-          <t>保留高浏览页面；对高跳出或低转化页面优化首屏价值、CTA和内部链接</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>2026-07-20</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>2026-07-26</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>/mg_proxy/home</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>Seeed Studio Bazaar, The IoT Hardware enabler.</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>8144</t>
-        </is>
-      </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>5168</t>
-        </is>
-      </c>
-      <c r="G11" t="inlineStr">
-        <is>
-          <t>5356</t>
-        </is>
-      </c>
-      <c r="H11" t="inlineStr">
-        <is>
-          <t>94.25%</t>
-        </is>
-      </c>
-      <c r="I11" t="inlineStr">
-        <is>
-          <t>5.75%</t>
-        </is>
-      </c>
-      <c r="J11" t="inlineStr">
-        <is>
-          <t>33.95</t>
-        </is>
-      </c>
-      <c r="K11" t="inlineStr">
-        <is>
-          <t>20</t>
-        </is>
-      </c>
-      <c r="L11" t="inlineStr">
-        <is>
-          <t>20</t>
-        </is>
-      </c>
-      <c r="M11" t="inlineStr">
-        <is>
-          <t>其他</t>
-        </is>
-      </c>
-      <c r="N11" t="inlineStr">
-        <is>
-          <t>转化偏弱，需检查表单、咨询入口和购买链路</t>
-        </is>
-      </c>
-      <c r="O11" t="inlineStr">
-        <is>
-          <t>保留高浏览页面；对高跳出或低转化页面优化首屏价值、CTA和内部链接</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>2026-07-20</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>2026-07-26</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>/XIAO-ESP32S3-Sense-p-5639.html</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>Mini ESP-CAM Dev Board for Edge AI - XIAO ESP32S3 Sense</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>7824</t>
-        </is>
-      </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>2880</t>
-        </is>
-      </c>
-      <c r="G12" t="inlineStr">
-        <is>
-          <t>3171</t>
-        </is>
-      </c>
-      <c r="H12" t="inlineStr">
-        <is>
-          <t>86.53%</t>
-        </is>
-      </c>
-      <c r="I12" t="inlineStr">
-        <is>
-          <t>13.47%</t>
-        </is>
-      </c>
-      <c r="J12" t="inlineStr">
-        <is>
-          <t>32.88</t>
-        </is>
-      </c>
-      <c r="K12" t="inlineStr">
-        <is>
-          <t>162</t>
-        </is>
-      </c>
-      <c r="L12" t="inlineStr">
-        <is>
-          <t>162</t>
-        </is>
-      </c>
-      <c r="M12" t="inlineStr">
-        <is>
-          <t>产品页</t>
-        </is>
-      </c>
-      <c r="N12" t="inlineStr">
-        <is>
-          <t>转化表现较强，可继续放大有效渠道</t>
-        </is>
-      </c>
-      <c r="O12" t="inlineStr">
-        <is>
-          <t>保留高浏览页面；对高跳出或低转化页面优化首屏价值、CTA和内部链接</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>2026-07-20</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>2026-07-26</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>/us_warehouse</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>US_Warehouse</t>
-        </is>
-      </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>7454</t>
-        </is>
-      </c>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>2904</t>
-        </is>
-      </c>
-      <c r="G13" t="inlineStr">
-        <is>
-          <t>3040</t>
-        </is>
-      </c>
-      <c r="H13" t="inlineStr">
-        <is>
-          <t>94.61%</t>
-        </is>
-      </c>
-      <c r="I13" t="inlineStr">
-        <is>
-          <t>5.39%</t>
-        </is>
-      </c>
-      <c r="J13" t="inlineStr">
-        <is>
-          <t>38.58</t>
-        </is>
-      </c>
-      <c r="K13" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="L13" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="M13" t="inlineStr">
-        <is>
-          <t>其他</t>
-        </is>
-      </c>
-      <c r="N13" t="inlineStr">
-        <is>
-          <t>转化偏弱，需检查表单、咨询入口和购买链路</t>
-        </is>
-      </c>
-      <c r="O13" t="inlineStr">
-        <is>
-          <t>保留高浏览页面；对高跳出或低转化页面优化首屏价值、CTA和内部链接</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>2026-07-20</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>2026-07-26</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>/XIAO-ESP32S3-p-5627.html</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>High-Performance Dev Board with Wi-Fi and BLE - XIAO ESP32S3</t>
-        </is>
-      </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>7250</t>
-        </is>
-      </c>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>2789</t>
-        </is>
-      </c>
-      <c r="G14" t="inlineStr">
-        <is>
-          <t>3043</t>
-        </is>
-      </c>
-      <c r="H14" t="inlineStr">
-        <is>
-          <t>85.90%</t>
-        </is>
-      </c>
-      <c r="I14" t="inlineStr">
-        <is>
-          <t>14.10%</t>
-        </is>
-      </c>
-      <c r="J14" t="inlineStr">
-        <is>
-          <t>29.28</t>
-        </is>
-      </c>
-      <c r="K14" t="inlineStr">
-        <is>
-          <t>90</t>
-        </is>
-      </c>
-      <c r="L14" t="inlineStr">
-        <is>
-          <t>90</t>
-        </is>
-      </c>
-      <c r="M14" t="inlineStr">
-        <is>
-          <t>产品页</t>
-        </is>
-      </c>
-      <c r="N14" t="inlineStr">
-        <is>
-          <t>转化处于可优化区间，建议做渠道和页面拆解</t>
-        </is>
-      </c>
-      <c r="O14" t="inlineStr">
-        <is>
-          <t>保留高浏览页面；对高跳出或低转化页面优化首屏价值、CTA和内部链接</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>2026-07-20</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>2026-07-26</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>/Grove-2-5A-DC-Current-Sensor-ACS70331-p-2929.html</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>Grove - 2.5A DC Current Sensor(ACS70331) - Seeed Studio</t>
-        </is>
-      </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>6716</t>
-        </is>
-      </c>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>3536</t>
-        </is>
-      </c>
-      <c r="G15" t="inlineStr">
-        <is>
-          <t>3537</t>
-        </is>
-      </c>
-      <c r="H15" t="inlineStr">
-        <is>
-          <t>90.05%</t>
-        </is>
-      </c>
-      <c r="I15" t="inlineStr">
-        <is>
-          <t>9.95%</t>
-        </is>
-      </c>
-      <c r="J15" t="inlineStr">
-        <is>
-          <t>1.58</t>
-        </is>
-      </c>
-      <c r="K15" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="L15" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="M15" t="inlineStr">
-        <is>
-          <t>产品页</t>
-        </is>
-      </c>
-      <c r="N15" t="inlineStr">
-        <is>
-          <t>转化偏弱，需检查表单、咨询入口和购买链路</t>
-        </is>
-      </c>
-      <c r="O15" t="inlineStr">
-        <is>
-          <t>保留高浏览页面；对高跳出或低转化页面优化首屏价值、CTA和内部链接</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>2026-07-20</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>2026-07-26</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>/reBot-Arm-B601-RS-Assembled-Kit-with-Gripper-p-6865.html</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>reBot Arm B601-RS : a low-cost 6-degree-of-freedom open-source robotic arm built based on the Lingzu Robstride series motors</t>
-        </is>
-      </c>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>6339</t>
-        </is>
-      </c>
-      <c r="F16" t="inlineStr">
-        <is>
-          <t>1831</t>
-        </is>
-      </c>
-      <c r="G16" t="inlineStr">
-        <is>
-          <t>1942</t>
-        </is>
-      </c>
-      <c r="H16" t="inlineStr">
-        <is>
-          <t>94.64%</t>
-        </is>
-      </c>
-      <c r="I16" t="inlineStr">
-        <is>
-          <t>5.36%</t>
-        </is>
-      </c>
-      <c r="J16" t="inlineStr">
-        <is>
-          <t>24.22</t>
-        </is>
-      </c>
-      <c r="K16" t="inlineStr">
-        <is>
-          <t>23</t>
-        </is>
-      </c>
-      <c r="L16" t="inlineStr">
-        <is>
-          <t>23</t>
-        </is>
-      </c>
-      <c r="M16" t="inlineStr">
-        <is>
-          <t>产品页</t>
-        </is>
-      </c>
-      <c r="N16" t="inlineStr">
-        <is>
-          <t>转化处于可优化区间，建议做渠道和页面拆解</t>
-        </is>
-      </c>
-      <c r="O16" t="inlineStr">
-        <is>
-          <t>保留高浏览页面；对高跳出或低转化页面优化首屏价值、CTA和内部链接</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>2026-07-20</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>2026-07-26</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>/TRMNL-7-5-Inch-OG-DIY-Kit-p-6481.html</t>
-        </is>
-      </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>TRMNL 7.5" DIY E-ink Dashboard Kit | Seeed Studio x TRMNL Official</t>
-        </is>
-      </c>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>5925</t>
-        </is>
-      </c>
-      <c r="F17" t="inlineStr">
-        <is>
-          <t>2147</t>
-        </is>
-      </c>
-      <c r="G17" t="inlineStr">
-        <is>
-          <t>2313</t>
-        </is>
-      </c>
-      <c r="H17" t="inlineStr">
-        <is>
-          <t>91.31%</t>
-        </is>
-      </c>
-      <c r="I17" t="inlineStr">
-        <is>
-          <t>8.69%</t>
-        </is>
-      </c>
-      <c r="J17" t="inlineStr">
-        <is>
-          <t>32.48</t>
-        </is>
-      </c>
-      <c r="K17" t="inlineStr">
-        <is>
-          <t>119</t>
-        </is>
-      </c>
-      <c r="L17" t="inlineStr">
-        <is>
-          <t>119</t>
-        </is>
-      </c>
-      <c r="M17" t="inlineStr">
-        <is>
-          <t>产品页</t>
-        </is>
-      </c>
-      <c r="N17" t="inlineStr">
-        <is>
-          <t>转化表现较强，可继续放大有效渠道</t>
-        </is>
-      </c>
-      <c r="O17" t="inlineStr">
-        <is>
-          <t>保留高浏览页面；对高跳出或低转化页面优化首屏价值、CTA和内部链接</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>2026-07-20</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>2026-07-26</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>/customer_order_shipment.html</t>
-        </is>
-      </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>Track Shipment</t>
-        </is>
-      </c>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>5738</t>
-        </is>
-      </c>
-      <c r="F18" t="inlineStr">
-        <is>
-          <t>2205</t>
-        </is>
-      </c>
-      <c r="G18" t="inlineStr">
-        <is>
-          <t>2844</t>
-        </is>
-      </c>
-      <c r="H18" t="inlineStr">
-        <is>
-          <t>81.50%</t>
-        </is>
-      </c>
-      <c r="I18" t="inlineStr">
-        <is>
-          <t>18.50%</t>
-        </is>
-      </c>
-      <c r="J18" t="inlineStr">
-        <is>
-          <t>13.63</t>
-        </is>
-      </c>
-      <c r="K18" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="L18" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="M18" t="inlineStr">
-        <is>
-          <t>产品页</t>
-        </is>
-      </c>
-      <c r="N18" t="inlineStr">
-        <is>
-          <t>转化偏弱，需检查表单、咨询入口和购买链路</t>
-        </is>
-      </c>
-      <c r="O18" t="inlineStr">
-        <is>
-          <t>保留高浏览页面；对高跳出或低转化页面优化首屏价值、CTA和内部链接</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>2026-07-20</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>2026-07-26</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>/Seeed-Studio-XIAO-ESP32C6-p-5884.html</t>
-        </is>
-      </c>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>Tiny Matter-Native Board for Smart Home - XIAO ESP32C6</t>
-        </is>
-      </c>
-      <c r="E19" t="inlineStr">
-        <is>
-          <t>5705</t>
-        </is>
-      </c>
-      <c r="F19" t="inlineStr">
-        <is>
-          <t>2002</t>
-        </is>
-      </c>
-      <c r="G19" t="inlineStr">
-        <is>
-          <t>2170</t>
-        </is>
-      </c>
-      <c r="H19" t="inlineStr">
-        <is>
-          <t>88.94%</t>
-        </is>
-      </c>
-      <c r="I19" t="inlineStr">
-        <is>
-          <t>11.06%</t>
-        </is>
-      </c>
-      <c r="J19" t="inlineStr">
-        <is>
-          <t>27.84</t>
-        </is>
-      </c>
-      <c r="K19" t="inlineStr">
-        <is>
-          <t>55</t>
-        </is>
-      </c>
-      <c r="L19" t="inlineStr">
-        <is>
-          <t>55</t>
-        </is>
-      </c>
-      <c r="M19" t="inlineStr">
-        <is>
-          <t>产品页</t>
-        </is>
-      </c>
-      <c r="N19" t="inlineStr">
-        <is>
-          <t>转化处于可优化区间，建议做渠道和页面拆解</t>
-        </is>
-      </c>
-      <c r="O19" t="inlineStr">
-        <is>
-          <t>保留高浏览页面；对高跳出或低转化页面优化首屏价值、CTA和内部链接</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>2026-07-20</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>2026-07-26</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>/reCamera-Pro-2GB.html</t>
-        </is>
-      </c>
-      <c r="D20" t="inlineStr">
-        <is>
-          <t>Edge AI Camera with Local AI Inference Seeed Studio</t>
-        </is>
-      </c>
-      <c r="E20" t="inlineStr">
-        <is>
-          <t>5661</t>
-        </is>
-      </c>
-      <c r="F20" t="inlineStr">
-        <is>
-          <t>1881</t>
-        </is>
-      </c>
-      <c r="G20" t="inlineStr">
-        <is>
-          <t>2084</t>
-        </is>
-      </c>
-      <c r="H20" t="inlineStr">
-        <is>
-          <t>89.59%</t>
-        </is>
-      </c>
-      <c r="I20" t="inlineStr">
-        <is>
-          <t>10.41%</t>
-        </is>
-      </c>
-      <c r="J20" t="inlineStr">
-        <is>
-          <t>52.17</t>
-        </is>
-      </c>
-      <c r="K20" t="inlineStr">
-        <is>
-          <t>42</t>
-        </is>
-      </c>
-      <c r="L20" t="inlineStr">
-        <is>
-          <t>42</t>
-        </is>
-      </c>
-      <c r="M20" t="inlineStr">
-        <is>
-          <t>产品页</t>
-        </is>
-      </c>
-      <c r="N20" t="inlineStr">
-        <is>
-          <t>转化处于可优化区间，建议做渠道和页面拆解</t>
-        </is>
-      </c>
-      <c r="O20" t="inlineStr">
-        <is>
-          <t>保留高浏览页面；对高跳出或低转化页面优化首屏价值、CTA和内部链接</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>2026-07-20</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>2026-07-26</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>/checkout/cart/</t>
-        </is>
-      </c>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>Seeed Studio Bazaar, The IoT Hardware enabler.</t>
-        </is>
-      </c>
-      <c r="E21" t="inlineStr">
-        <is>
-          <t>5496</t>
-        </is>
-      </c>
-      <c r="F21" t="inlineStr">
-        <is>
-          <t>1313</t>
-        </is>
-      </c>
-      <c r="G21" t="inlineStr">
-        <is>
-          <t>1374</t>
-        </is>
-      </c>
-      <c r="H21" t="inlineStr">
-        <is>
-          <t>97.31%</t>
-        </is>
-      </c>
-      <c r="I21" t="inlineStr">
-        <is>
-          <t>2.69%</t>
-        </is>
-      </c>
-      <c r="J21" t="inlineStr">
-        <is>
-          <t>15.16</t>
-        </is>
-      </c>
-      <c r="K21" t="inlineStr">
-        <is>
-          <t>20</t>
-        </is>
-      </c>
-      <c r="L21" t="inlineStr">
-        <is>
-          <t>20</t>
-        </is>
-      </c>
-      <c r="M21" t="inlineStr">
-        <is>
-          <t>购买/购物车</t>
-        </is>
-      </c>
-      <c r="N21" t="inlineStr">
-        <is>
-          <t>转化处于可优化区间，建议做渠道和页面拆解</t>
-        </is>
-      </c>
-      <c r="O21" t="inlineStr">
         <is>
           <t>保留高浏览页面；对高跳出或低转化页面优化首屏价值、CTA和内部链接</t>
         </is>
@@ -2981,22 +1826,22 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>3422</t>
+          <t>0</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>3226</t>
+          <t>0</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>179</t>
+          <t>0</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>5.23%</t>
+          <t>0.00%</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">

</xml_diff>